<commit_message>
fix runq3 and the core logic of mpc q3
</commit_message>
<xml_diff>
--- a/results/q3_summary.xlsx
+++ b/results/q3_summary.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,12 +417,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -447,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>22587503.7</v>
+        <v>24712006.22</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +445,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22652359.6</v>
+        <v>24812775.48</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>230806.32</v>
+        <v>57042.44</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17586537.22</v>
+        <v>15426704.49</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +475,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44115.98</v>
+        <v>134734.28</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +485,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1023283.99</v>
+        <v>308139.55</v>
       </c>
     </row>
     <row r="8">
@@ -507,7 +495,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18653937.18</v>
+        <v>15869578.32</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +505,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>178110.28</v>
+        <v>215832.11</v>
       </c>
     </row>
     <row r="10">
@@ -527,7 +515,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.95</v>
+        <v>1.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor Q3 MPC per spec and regenerate Q3 results
</commit_message>
<xml_diff>
--- a/results/q3_summary.xlsx
+++ b/results/q3_summary.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,12 +429,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -435,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24712006.22</v>
+        <v>21406733.46</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24812775.48</v>
+        <v>22268064.46</v>
       </c>
     </row>
     <row r="4">
@@ -455,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>57042.44</v>
+        <v>833074.22</v>
       </c>
     </row>
     <row r="5">
@@ -465,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15426704.49</v>
+        <v>12647020.99</v>
       </c>
     </row>
     <row r="6">
@@ -475,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>134734.28</v>
+        <v>1869229.5</v>
       </c>
     </row>
     <row r="7">
@@ -485,7 +497,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>308139.55</v>
+        <v>4728044.33</v>
       </c>
     </row>
     <row r="8">
@@ -495,27 +507,27 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15869578.32</v>
+        <v>19244294.82</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cost Reduction vs Q2 (Yuan)</t>
+          <t>Cost Reduction vs Q2 Baseline (Yuan)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>215832.11</v>
+        <v>-412247.36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cost Reduction vs Q2 (%)</t>
+          <t>Cost Reduction vs Q2 Baseline (%)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.34</v>
+        <v>-2.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
optimized q2 q3 and q4
</commit_message>
<xml_diff>
--- a/results/q3_summary.xlsx
+++ b/results/q3_summary.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,12 +417,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -447,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>21406733.46</v>
+        <v>26160203</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +445,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22268064.46</v>
+        <v>25775995.73</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>833074.22</v>
+        <v>89266.72</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12647020.99</v>
+        <v>16393170.77</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +475,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1869229.5</v>
+        <v>768556.16</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +485,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4728044.33</v>
+        <v>455381.82</v>
       </c>
     </row>
     <row r="8">
@@ -507,7 +495,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19244294.82</v>
+        <v>17617108.75</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +505,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-412247.36</v>
+        <v>1214938.71</v>
       </c>
     </row>
     <row r="10">
@@ -527,7 +515,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-2.19</v>
+        <v>6.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revised Q3 and Q4
</commit_message>
<xml_diff>
--- a/results/q3_summary.xlsx
+++ b/results/q3_summary.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,16 +425,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -435,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>26160203</v>
+        <v>24719291.25</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25775995.73</v>
+        <v>24282953.59</v>
       </c>
     </row>
     <row r="4">
@@ -455,67 +467,99 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>89266.72</v>
+        <v>47213.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Baseline Purchase Cost (Yuan)</t>
+          <t>Q2 Optimized Baseline Cost (Yuan)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16393170.77</v>
+        <v>16085410.43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Adjustment Surcharge/Breach Cost (Yuan)</t>
+          <t>Baseline Purchase Cost (Yuan)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>768556.16</v>
+        <v>18832047.46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Emergency Penalty Cost (Yuan)</t>
+          <t>Adjustment Surcharge/Breach Cost (Yuan)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>455381.82</v>
+        <v>189028.99</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Total Settlement Cost Q3 (Yuan)</t>
+          <t>Emergency Penalty Cost (Yuan)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17617108.75</v>
+        <v>248777.28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cost Reduction vs Q2 Baseline (Yuan)</t>
+          <t>Total Settlement Cost Q3 (Yuan)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1214938.71</v>
+        <v>15867644.03</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cost Reduction vs Q2 Baseline (%)</t>
+          <t>Cost Reduction vs Heuristic Baseline (Yuan)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.45</v>
+        <v>2964403.43</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cost Reduction vs Heuristic Baseline (%)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>15.74</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cost Reduction vs Q2 Optimized (Yuan)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>217766.4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Monotonicity C_Q1 &lt;= C_Q3 &lt; C_Q2 &lt; C_Baseline</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>